<commit_message>
Creation of calibration streamlit interface
</commit_message>
<xml_diff>
--- a/001_output/df_yr1_001.xlsx
+++ b/001_output/df_yr1_001.xlsx
@@ -1,20 +1,63 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nv5inc-my.sharepoint.com/personal/andrewj_johnson_nv5_com/Documents/Documents/GitHub/Potential_Study_Tool_Prototype/001_output/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_23F921EDAB6BCCFDE32354B62176E7747452BD27" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{528DC37F-885F-47DE-A0A8-C2D68B63402C}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="28680" yWindow="-3420" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="37">
   <si>
     <t>competition_group</t>
   </si>
@@ -98,13 +141,40 @@
   </si>
   <si>
     <t>none</t>
+  </si>
+  <si>
+    <t>condition_name</t>
+  </si>
+  <si>
+    <t>whole_home_natural_gas_baseline_residential</t>
+  </si>
+  <si>
+    <t>insulation_natural_gas_efficient_residential</t>
+  </si>
+  <si>
+    <t>HERS_electricity_efficient_residential</t>
+  </si>
+  <si>
+    <t>room_ac_electricity_baseline_residential</t>
+  </si>
+  <si>
+    <t>room_ac_electricity_efficient_residential</t>
+  </si>
+  <si>
+    <t>air_conditioner_electricity_baseline_residential</t>
+  </si>
+  <si>
+    <t>cchp_electricity_efficient_residential</t>
+  </si>
+  <si>
+    <t>air_conditioner_electricity_efficient_residential</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -119,6 +189,11 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -156,9 +231,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
@@ -167,13 +245,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -211,7 +297,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -245,6 +331,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -279,9 +366,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -454,11 +542,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:K31"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="15.28515625" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="3" max="3" width="21.7109375" customWidth="1"/>
+    <col min="4" max="4" width="43.140625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -490,7 +584,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -525,7 +619,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -560,7 +654,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -595,7 +689,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -630,7 +724,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -665,7 +759,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -700,7 +794,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -735,7 +829,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="9" spans="1:11">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -770,7 +864,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="10" spans="1:11">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -805,7 +899,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -840,7 +934,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="12" spans="1:11">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -875,7 +969,7 @@
         <v>1000</v>
       </c>
     </row>
-    <row r="13" spans="1:11">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -910,7 +1004,7 @@
         <v>700</v>
       </c>
     </row>
-    <row r="14" spans="1:11">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>12</v>
       </c>
@@ -945,7 +1039,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="15" spans="1:11">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -980,7 +1074,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="16" spans="1:11">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -1015,7 +1109,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -1050,7 +1144,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -1085,7 +1179,7 @@
         <v>500</v>
       </c>
     </row>
-    <row r="19" spans="1:11">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -1120,7 +1214,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -1155,7 +1249,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -1190,7 +1284,7 @@
         <v>6000</v>
       </c>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>20</v>
       </c>
@@ -1225,7 +1319,7 @@
         <v>4200</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -1260,7 +1354,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -1295,7 +1389,7 @@
         <v>6000</v>
       </c>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -1330,7 +1424,7 @@
         <v>4200</v>
       </c>
     </row>
-    <row r="26" spans="1:11">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -1365,7 +1459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:11">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -1400,7 +1494,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:11">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -1435,7 +1529,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:11">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>27</v>
       </c>
@@ -1470,7 +1564,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:11">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>28</v>
       </c>
@@ -1505,7 +1599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:11">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>29</v>
       </c>
@@ -1538,6 +1632,867 @@
       </c>
       <c r="K31">
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A828483D-BED1-4390-8CAA-E74484F28A96}">
+  <dimension ref="A1:D135"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="44.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" t="str" cm="1">
+        <f t="array" ref="D1:D17">_xlfn.UNIQUE(A:A)</f>
+        <v>condition_name</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D2" t="str">
+        <v>furnace_oil_existing_residential</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" t="str">
+        <v>whole_home_natural_gas_baseline_residential</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" t="str">
+        <v>insulation_natural_gas_efficient_residential</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="str">
+        <v>HERS_electricity_efficient_residential</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="str">
+        <v>furnace_natural_gas_baseline_residential</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" t="str">
+        <v>furnace_natural_gas_efficient_residential</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" t="str">
+        <v>room_ac_electricity_baseline_residential</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" t="str">
+        <v>room_ac_electricity_efficient_residential</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D10" t="str">
+        <v>air_conditioner_electricity_baseline_residential</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>29</v>
+      </c>
+      <c r="D11" t="str">
+        <v>cchp_electricity_efficient_residential</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" t="str">
+        <v>air_conditioner_electricity_efficient_residential</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" t="str">
+        <v>refrigerator_electricity_existing_residential</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>29</v>
+      </c>
+      <c r="D14" t="str">
+        <v>refrigerator_electricity_baseline_residential</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" t="str">
+        <v>refrigerator_electricity_efficient_residential</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" t="str">
+        <v>refrigerator_electricity_top10_residential</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="97" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="98" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="99" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="100" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="101" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="102" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="103" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="104" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A104" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="105" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A105" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="106" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A106" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="107" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A107" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="108" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="109" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="110" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="111" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="112" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="113" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="114" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="115" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="116" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="117" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="118" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="119" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="120" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="121" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="122" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="123" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="124" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="125" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="126" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="127" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="128" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>23</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B5EFDC6-04FC-4604-9913-DCC6A245E38A}">
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18.42578125" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C2" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C3" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C4" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C14" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C15" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C16" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>